<commit_message>
feat: preserve local automation and Excel changes
</commit_message>
<xml_diff>
--- a/test_cases/test_case.xlsx
+++ b/test_cases/test_case.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="17655" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="自动化测试用例" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,14 +12,14 @@
     <sheet name="操作类型说明" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="12">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -60,114 +60,36 @@
     <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
+      <family val="3"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <color rgb="FF800080"/>
+      <family val="3"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="宋体"/>
       <charset val="134"/>
       <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
       <color rgb="FF9C0006"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <color rgb="FF9C6500"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <color theme="0"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FF9C0006"/>
     </font>
     <font/>
   </fonts>
-  <fills count="38">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -206,192 +128,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39998"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -414,253 +156,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.49998"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -677,7 +177,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -687,74 +186,148 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.7999511703848384"/>
+          <bgColor theme="4" tint="0.7999511703848384"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.3999450666829432"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.7999511703848384"/>
+          <bgColor theme="4" tint="0.7999511703848384"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.3999450666829432"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.3999450666829432"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.7999511703848384"/>
+          <bgColor theme="4" tint="0.7999511703848384"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.7999511703848384"/>
+          <bgColor theme="4" tint="0.7999511703848384"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.7999511703848384"/>
+          <bgColor theme="4" tint="0.7999511703848384"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.3999450666829432"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.3999450666829432"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.7999511703848384"/>
+          <bgColor theme="4" tint="0.7999511703848384"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.3999450666829432"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.7999511703848384"/>
+          <bgColor theme="4" tint="0.7999511703848384"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.7999511703848384"/>
+          <bgColor theme="4" tint="0.7999511703848384"/>
         </patternFill>
       </fill>
     </dxf>
@@ -811,149 +384,32 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.3999450666829432"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1237,6 +693,7 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -1247,9 +704,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R123"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="25.8416666666667" customWidth="1" min="1" max="1"/>
+    <col width="25.81640625" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -1264,7 +721,7 @@
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="14.5" customWidth="1" min="17" max="17"/>
+    <col width="14.453125" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1360,7 +817,7 @@
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>TC-LOGIN-001</t>
         </is>
@@ -1439,7 +896,7 @@
           <t>错误账号测试</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="Q2" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1531,7 +988,7 @@
           <t>错误密码测试</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="Q3" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1617,7 +1074,7 @@
           <t>必填校验</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="Q4" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1704,7 +1161,7 @@
       <c r="O5" t="n">
         <v>3</v>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="Q5" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1792,7 +1249,7 @@
       <c r="O6" t="n">
         <v>3</v>
       </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="Q6" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1873,7 +1330,7 @@
       <c r="O7" t="n">
         <v>3</v>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
+      <c r="Q7" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1966,7 +1423,7 @@
           <t>正常登录流程</t>
         </is>
       </c>
-      <c r="Q8" s="3" t="inlineStr">
+      <c r="Q8" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2046,7 +1503,7 @@
       <c r="O9" t="n">
         <v>5</v>
       </c>
-      <c r="Q9" s="3" t="inlineStr">
+      <c r="Q9" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2132,7 +1589,7 @@
       <c r="O10" t="n">
         <v>5</v>
       </c>
-      <c r="Q10" s="3" t="inlineStr">
+      <c r="Q10" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2143,85 +1600,85 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="28" customFormat="1" customHeight="1" s="4">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>TC-HOME-003</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>首页搜索</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>搜索-不存在的手机号</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>验证无结果提示</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>p1</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>已登录成功</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>1.在搜索框输入不存在的手机号
 2.点击搜索</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>input[placeholder='请输入关键字'], button:has-text('搜 索')</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>input,click</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>13626710399</v>
-      </c>
-      <c r="K11" t="inlineStr">
+      <c r="J11" s="18" t="n">
+        <v>100000000000</v>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>展示：暂无内容</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>页面显示'暂无'</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>text_visible</t>
         </is>
       </c>
-      <c r="O11" t="n">
+      <c r="O11" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="Q11" s="3" t="inlineStr">
+      <c r="Q11" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="R11" s="4" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -2274,7 +1731,7 @@
           <t>input,click</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="15" t="inlineStr">
         <is>
           <t>t</t>
         </is>
@@ -2302,7 +1759,7 @@
       <c r="O12" t="n">
         <v>5</v>
       </c>
-      <c r="Q12" s="3" t="inlineStr">
+      <c r="Q12" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2388,7 +1845,7 @@
       <c r="O13" t="n">
         <v>5</v>
       </c>
-      <c r="Q13" s="3" t="inlineStr">
+      <c r="Q13" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2472,7 +1929,7 @@
       <c r="O14" t="n">
         <v>5</v>
       </c>
-      <c r="Q14" s="3" t="inlineStr">
+      <c r="Q14" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2556,7 +2013,7 @@
       <c r="O15" t="n">
         <v>5</v>
       </c>
-      <c r="Q15" s="3" t="inlineStr">
+      <c r="Q15" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2636,7 +2093,7 @@
       <c r="O16" t="n">
         <v>5</v>
       </c>
-      <c r="Q16" s="3" t="inlineStr">
+      <c r="Q16" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2716,7 +2173,7 @@
       <c r="O17" t="n">
         <v>5</v>
       </c>
-      <c r="Q17" s="3" t="inlineStr">
+      <c r="Q17" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2796,7 +2253,7 @@
       <c r="O18" t="n">
         <v>5</v>
       </c>
-      <c r="Q18" s="3" t="inlineStr">
+      <c r="Q18" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2876,7 +2333,7 @@
       <c r="O19" t="n">
         <v>5</v>
       </c>
-      <c r="Q19" s="3" t="inlineStr">
+      <c r="Q19" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2956,7 +2413,7 @@
       <c r="O20" t="n">
         <v>15</v>
       </c>
-      <c r="Q20" s="3" t="inlineStr">
+      <c r="Q20" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3037,7 +2494,7 @@
       <c r="O21" t="n">
         <v>10</v>
       </c>
-      <c r="Q21" s="3" t="inlineStr">
+      <c r="Q21" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3118,7 +2575,7 @@
       <c r="O22" t="n">
         <v>10</v>
       </c>
-      <c r="Q22" s="3" t="inlineStr">
+      <c r="Q22" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3199,7 +2656,7 @@
       <c r="O23" t="n">
         <v>10</v>
       </c>
-      <c r="Q23" s="3" t="inlineStr">
+      <c r="Q23" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3210,82 +2667,82 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" t="inlineStr">
+    <row r="24" ht="28" customFormat="1" customHeight="1" s="4">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>TC-CUSTOMER-004</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>顾客列表</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>搜索-不存在的手机号</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>验证无结果提示</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>已登录并进入顾客列表页</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="G24" s="13" t="inlineStr">
         <is>
           <t>1.在搜索框输入不存在的手机号
 2.点击搜索</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>/customer, 0.5, input[placeholder='请输入关键字'], button:has-text('搜 索')</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>nav, wait, input, click</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>|13626710399</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
+      <c r="J24" s="18" t="inlineStr">
+        <is>
+          <t>|100000000000</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>展示：暂无内容</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>'暂无'</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>text_visible</t>
         </is>
       </c>
-      <c r="O24" t="n">
+      <c r="O24" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q24" s="3" t="inlineStr">
+      <c r="Q24" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="R24" s="4" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -3361,7 +2818,7 @@
       <c r="O25" t="n">
         <v>10</v>
       </c>
-      <c r="Q25" s="3" t="inlineStr">
+      <c r="Q25" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3442,7 +2899,7 @@
       <c r="O26" t="n">
         <v>10</v>
       </c>
-      <c r="Q26" s="3" t="inlineStr">
+      <c r="Q26" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3523,7 +2980,7 @@
       <c r="O27" t="n">
         <v>5</v>
       </c>
-      <c r="Q27" s="3" t="inlineStr">
+      <c r="Q27" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3608,7 +3065,7 @@
       <c r="O28" t="n">
         <v>5</v>
       </c>
-      <c r="Q28" s="3" t="inlineStr">
+      <c r="Q28" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3689,7 +3146,7 @@
       <c r="O29" t="n">
         <v>5</v>
       </c>
-      <c r="Q29" s="3" t="inlineStr">
+      <c r="Q29" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3775,7 +3232,7 @@
       <c r="O30" t="n">
         <v>10</v>
       </c>
-      <c r="Q30" s="3" t="inlineStr">
+      <c r="Q30" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3861,7 +3318,7 @@
       <c r="O31" t="n">
         <v>10</v>
       </c>
-      <c r="Q31" s="3" t="inlineStr">
+      <c r="Q31" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3950,7 +3407,7 @@
       <c r="O32" t="n">
         <v>10</v>
       </c>
-      <c r="Q32" s="3" t="inlineStr">
+      <c r="Q32" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4039,7 +3496,7 @@
       <c r="O33" t="n">
         <v>10</v>
       </c>
-      <c r="Q33" s="3" t="inlineStr">
+      <c r="Q33" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4128,7 +3585,7 @@
       <c r="O34" t="n">
         <v>10</v>
       </c>
-      <c r="Q34" s="3" t="inlineStr">
+      <c r="Q34" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4217,7 +3674,7 @@
       <c r="O35" t="n">
         <v>10</v>
       </c>
-      <c r="Q35" s="3" t="inlineStr">
+      <c r="Q35" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4306,7 +3763,7 @@
       <c r="O36" t="n">
         <v>10</v>
       </c>
-      <c r="Q36" s="3" t="inlineStr">
+      <c r="Q36" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4395,7 +3852,7 @@
       <c r="O37" t="n">
         <v>10</v>
       </c>
-      <c r="Q37" s="3" t="inlineStr">
+      <c r="Q37" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4471,7 +3928,7 @@
           <t>展示符合时间范围的顾客档案</t>
         </is>
       </c>
-      <c r="M38" s="15" t="inlineStr">
+      <c r="M38" s="14" t="inlineStr">
         <is>
           <t>'详情'</t>
         </is>
@@ -4484,7 +3941,7 @@
       <c r="O38" t="n">
         <v>10</v>
       </c>
-      <c r="Q38" s="3" t="inlineStr">
+      <c r="Q38" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4562,7 +4019,7 @@
           <t>已根据实际DOM调整：删除'已为'步骤；确定按钮用.ant-popover .ant-btn-primary；备注图标用.ant-image + div .anticon</t>
         </is>
       </c>
-      <c r="Q39" s="3" t="inlineStr">
+      <c r="Q39" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4648,7 +4105,7 @@
           <t>卡片为自定义结构（非ant-list）；性别图标为图片形式无法文本断言；字段验证：姓名/年龄/手机号/上次检测时间/检测次数/详情</t>
         </is>
       </c>
-      <c r="Q40" s="3" t="inlineStr">
+      <c r="Q40" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4728,7 +4185,7 @@
       <c r="O41" t="n">
         <v>5</v>
       </c>
-      <c r="Q41" s="3" t="inlineStr">
+      <c r="Q41" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4810,7 +4267,7 @@
       <c r="O42" t="n">
         <v>10</v>
       </c>
-      <c r="Q42" s="3" t="inlineStr">
+      <c r="Q42" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4893,7 +4350,7 @@
       <c r="O43" t="n">
         <v>3</v>
       </c>
-      <c r="Q43" s="3" t="inlineStr">
+      <c r="Q43" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5071,7 +4528,7 @@
       <c r="O45" t="n">
         <v>10</v>
       </c>
-      <c r="Q45" s="3" t="inlineStr">
+      <c r="Q45" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5159,7 +4616,7 @@
       <c r="O46" t="n">
         <v>10</v>
       </c>
-      <c r="Q46" s="3" t="inlineStr">
+      <c r="Q46" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5247,7 +4704,7 @@
       <c r="O47" t="n">
         <v>10</v>
       </c>
-      <c r="Q47" s="3" t="inlineStr">
+      <c r="Q47" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5322,7 +4779,7 @@
           <t>保存成功，性别显示'保密'</t>
         </is>
       </c>
-      <c r="M48" s="15" t="inlineStr">
+      <c r="M48" s="14" t="inlineStr">
         <is>
           <t>'性别下拉显示保密'</t>
         </is>
@@ -5335,7 +4792,7 @@
       <c r="O48" t="n">
         <v>15</v>
       </c>
-      <c r="Q48" s="3" t="inlineStr">
+      <c r="Q48" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5418,7 +4875,7 @@
       <c r="O49" t="n">
         <v>15</v>
       </c>
-      <c r="Q49" s="3" t="inlineStr">
+      <c r="Q49" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5501,7 +4958,7 @@
           <t>清空家庭住址后保存</t>
         </is>
       </c>
-      <c r="Q50" s="3" t="inlineStr">
+      <c r="Q50" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5589,7 +5046,7 @@
           <t>家庭住址输入特殊字符后保存</t>
         </is>
       </c>
-      <c r="Q51" s="3" t="inlineStr">
+      <c r="Q51" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5672,7 +5129,7 @@
           <t>家庭住址输入空格后保存</t>
         </is>
       </c>
-      <c r="Q52" s="3" t="inlineStr">
+      <c r="Q52" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5754,7 +5211,7 @@
       <c r="O53" t="n">
         <v>3</v>
       </c>
-      <c r="Q53" s="3" t="inlineStr">
+      <c r="Q53" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5843,7 +5300,7 @@
       <c r="O54" t="n">
         <v>5</v>
       </c>
-      <c r="Q54" s="3" t="inlineStr">
+      <c r="Q54" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5926,7 +5383,7 @@
           <t>清空备注后保存，备注非必填</t>
         </is>
       </c>
-      <c r="Q55" s="3" t="inlineStr">
+      <c r="Q55" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6014,7 +5471,7 @@
           <t>备注输入特殊字符后保存</t>
         </is>
       </c>
-      <c r="Q56" s="3" t="inlineStr">
+      <c r="Q56" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6092,7 +5549,7 @@
       <c r="O57" t="n">
         <v>10</v>
       </c>
-      <c r="Q57" s="3" t="inlineStr">
+      <c r="Q57" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6165,7 +5622,7 @@
           <t>最新保存的标签在最前面展示</t>
         </is>
       </c>
-      <c r="M58" s="15" t="inlineStr">
+      <c r="M58" s="14" t="inlineStr">
         <is>
           <t>'自动化标签测试1'</t>
         </is>
@@ -6183,7 +5640,7 @@
           <t>nav进入顾客列表，影像编辑图标易缺失，因此改为更稳妥的div</t>
         </is>
       </c>
-      <c r="Q58" s="3" t="inlineStr">
+      <c r="Q58" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6264,7 +5721,7 @@
       <c r="O59" t="n">
         <v>15</v>
       </c>
-      <c r="Q59" s="3" t="inlineStr">
+      <c r="Q59" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6355,7 +5812,7 @@
           <t>nav改为div,输入注意去掉占位符，否则读取不到</t>
         </is>
       </c>
-      <c r="Q60" s="3" t="inlineStr">
+      <c r="Q60" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6436,7 +5893,7 @@
       <c r="O61" t="n">
         <v>15</v>
       </c>
-      <c r="Q61" s="3" t="inlineStr">
+      <c r="Q61" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6521,7 +5978,7 @@
           <t>标签「自动化标签测试1」需已存在（由 TC-DETAIL-016 生成）</t>
         </is>
       </c>
-      <c r="Q62" s="3" t="inlineStr">
+      <c r="Q62" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6611,7 +6068,7 @@
           <t>需要有历史影像</t>
         </is>
       </c>
-      <c r="Q63" s="3" t="inlineStr">
+      <c r="Q63" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6696,7 +6153,7 @@
       <c r="O64" t="n">
         <v>15</v>
       </c>
-      <c r="Q64" s="3" t="inlineStr">
+      <c r="Q64" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6781,7 +6238,7 @@
           <t>需要有历史影像</t>
         </is>
       </c>
-      <c r="Q65" s="3" t="inlineStr">
+      <c r="Q65" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6865,7 +6322,7 @@
           <t>需要有历史影像；验证管理/完成按钮来回切换</t>
         </is>
       </c>
-      <c r="Q66" s="3" t="inlineStr">
+      <c r="Q66" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7043,7 +6500,7 @@
       <c r="O68" t="n">
         <v>15</v>
       </c>
-      <c r="Q68" s="3" t="inlineStr">
+      <c r="Q68" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7294,7 +6751,7 @@
           <t>需要有历史影像；管理模式下不选影像直接删除应提示</t>
         </is>
       </c>
-      <c r="Q71" s="3" t="inlineStr">
+      <c r="Q71" s="17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7336,7 +6793,7 @@
           <t>已登录，进入顾客列表页</t>
         </is>
       </c>
-      <c r="G72" s="11" t="inlineStr">
+      <c r="G72" s="10" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.在搜索框搜索咨询单特定用户
@@ -7362,7 +6819,6 @@
           <t>咨询单特定</t>
         </is>
       </c>
-      <c r="K72" s="3" t="n"/>
       <c r="L72" s="3" t="inlineStr">
         <is>
           <t>诊断结果下方出现最新创建的咨询单</t>
@@ -7386,7 +6842,7 @@
           <t>需要「咨询单特定」测试用户存在且有历史影像</t>
         </is>
       </c>
-      <c r="Q72" s="3" t="inlineStr">
+      <c r="Q72" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7428,7 +6884,7 @@
           <t>已登录，进入顾客列表页</t>
         </is>
       </c>
-      <c r="G73" s="11" t="inlineStr">
+      <c r="G73" s="10" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.在搜索框搜索咨询单特定用户
@@ -7454,7 +6910,6 @@
           <t>咨询单特定|咨询单标签测试</t>
         </is>
       </c>
-      <c r="K73" s="3" t="n"/>
       <c r="L73" s="3" t="inlineStr">
         <is>
           <t>标签页出现咨询单标签测试</t>
@@ -7478,7 +6933,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单；咨询单记录在诊断结果标签页</t>
         </is>
       </c>
-      <c r="Q73" s="3" t="inlineStr">
+      <c r="Q73" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7520,7 +6975,7 @@
           <t>已登录，进入顾客列表页</t>
         </is>
       </c>
-      <c r="G74" s="11" t="inlineStr">
+      <c r="G74" s="10" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.在搜索框搜索咨询单特定用户
@@ -7569,7 +7024,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q74" s="3" t="inlineStr">
+      <c r="Q74" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7611,7 +7066,7 @@
           <t>已登录，进入顾客列表页</t>
         </is>
       </c>
-      <c r="G75" s="11" t="inlineStr">
+      <c r="G75" s="10" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.在搜索框搜索咨询单特定用户
@@ -7660,7 +7115,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q75" s="3" t="inlineStr">
+      <c r="Q75" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7702,7 +7157,7 @@
           <t>已登录，进入顾客列表页</t>
         </is>
       </c>
-      <c r="G76" s="11" t="inlineStr">
+      <c r="G76" s="10" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.在搜索框搜索咨询单特定用户
@@ -7751,7 +7206,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q76" s="3" t="inlineStr">
+      <c r="Q76" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7793,7 +7248,7 @@
           <t>已登录，进入顾客列表页</t>
         </is>
       </c>
-      <c r="G77" s="11" t="inlineStr">
+      <c r="G77" s="10" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.在搜索框搜索咨询单特定用户
@@ -7841,7 +7296,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q77" s="3" t="inlineStr">
+      <c r="Q77" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7883,7 +7338,7 @@
           <t>已登录，进入顾客列表页</t>
         </is>
       </c>
-      <c r="G78" s="11" t="inlineStr">
+      <c r="G78" s="10" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.在搜索框搜索咨询单特定用户
@@ -7931,7 +7386,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q78" s="3" t="inlineStr">
+      <c r="Q78" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7973,7 +7428,7 @@
           <t>已登录，进入顾客列表页</t>
         </is>
       </c>
-      <c r="G79" s="11" t="inlineStr">
+      <c r="G79" s="10" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.在搜索框搜索咨询单特定用户
@@ -8023,7 +7478,7 @@
           <t>自包含用例：先新增固定备注再删除，验证点固定无需随测试数据更新</t>
         </is>
       </c>
-      <c r="Q79" s="3" t="inlineStr">
+      <c r="Q79" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8108,7 +7563,7 @@
       <c r="O80" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q80" s="12" t="inlineStr">
+      <c r="Q80" s="11" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8193,7 +7648,7 @@
       <c r="O81" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q81" s="12" t="inlineStr">
+      <c r="Q81" s="11" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8278,7 +7733,7 @@
       <c r="O82" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q82" s="12" t="inlineStr">
+      <c r="Q82" s="11" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8363,7 +7818,7 @@
       <c r="O83" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q83" s="13" t="inlineStr">
+      <c r="Q83" s="12" t="inlineStr">
         <is>
           <t>fail: utils\step_executor.py:170: in _do_click
     element.click(force=True, timeout=self.timeout_ms)
@@ -8453,7 +7908,7 @@
       <c r="O84" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q84" s="13" t="inlineStr">
+      <c r="Q84" s="12" t="inlineStr">
         <is>
           <t>fail: utils\step_executor.py:170: in _do_click
     element.click(force=True, timeout=self.timeout_ms)
@@ -8538,7 +7993,7 @@
       <c r="O85" t="n">
         <v>5</v>
       </c>
-      <c r="Q85" s="3" t="inlineStr">
+      <c r="Q85" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8623,7 +8078,7 @@
       <c r="O86" t="n">
         <v>5</v>
       </c>
-      <c r="Q86" s="3" t="inlineStr">
+      <c r="Q86" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8708,7 +8163,7 @@
       <c r="O87" t="n">
         <v>5</v>
       </c>
-      <c r="Q87" s="3" t="inlineStr">
+      <c r="Q87" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8788,7 +8243,7 @@
       <c r="O88" t="n">
         <v>5</v>
       </c>
-      <c r="Q88" s="3" t="inlineStr">
+      <c r="Q88" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8958,7 +8413,7 @@
       <c r="O90" t="n">
         <v>3</v>
       </c>
-      <c r="Q90" s="3" t="inlineStr">
+      <c r="Q90" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9044,7 +8499,7 @@
       <c r="O91" t="n">
         <v>3</v>
       </c>
-      <c r="Q91" s="3" t="inlineStr">
+      <c r="Q91" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9130,7 +8585,7 @@
       <c r="O92" t="n">
         <v>3</v>
       </c>
-      <c r="Q92" s="3" t="inlineStr">
+      <c r="Q92" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9216,7 +8671,7 @@
       <c r="O93" t="n">
         <v>3</v>
       </c>
-      <c r="Q93" s="3" t="inlineStr">
+      <c r="Q93" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9228,7 +8683,7 @@
       </c>
     </row>
     <row r="94" ht="28" customFormat="1" customHeight="1" s="4">
-      <c r="G94" s="14" t="n"/>
+      <c r="G94" s="13" t="n"/>
     </row>
     <row r="95" ht="28" customFormat="1" customHeight="1" s="4">
       <c r="A95" s="4" t="inlineStr">
@@ -9313,7 +8768,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q95" s="12" t="inlineStr">
+      <c r="Q95" s="11" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9407,7 +8862,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q96" s="12" t="inlineStr">
+      <c r="Q96" s="11" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9501,7 +8956,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q97" s="4" t="n"/>
       <c r="R97" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -9591,7 +9045,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q98" s="4" t="n"/>
       <c r="R98" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -9629,7 +9082,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G99" s="14" t="inlineStr">
+      <c r="G99" s="13" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -9681,7 +9134,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q99" s="4" t="n"/>
       <c r="R99" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -9719,7 +9171,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G100" s="14" t="inlineStr">
+      <c r="G100" s="13" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -9771,7 +9223,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q100" s="4" t="n"/>
       <c r="R100" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -9809,7 +9260,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G101" s="14" t="inlineStr">
+      <c r="G101" s="13" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -9861,7 +9312,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q101" s="4" t="n"/>
       <c r="R101" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -9951,7 +9401,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q102" s="12" t="inlineStr">
+      <c r="Q102" s="11" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -10045,7 +9495,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q103" s="4" t="n"/>
       <c r="R103" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10135,7 +9584,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q104" s="4" t="n"/>
       <c r="R104" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10225,7 +9673,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q105" s="4" t="n"/>
       <c r="R105" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10315,7 +9762,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q106" s="4" t="n"/>
       <c r="R106" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10405,7 +9851,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q107" s="4" t="n"/>
       <c r="R107" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10443,7 +9888,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G108" s="14" t="inlineStr">
+      <c r="G108" s="13" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -10495,7 +9940,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q108" s="4" t="n"/>
       <c r="R108" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10533,7 +9977,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G109" s="14" t="inlineStr">
+      <c r="G109" s="13" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -10585,7 +10029,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q109" s="4" t="n"/>
       <c r="R109" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10675,7 +10118,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q110" s="4" t="n"/>
       <c r="R110" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10713,7 +10155,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G111" s="14" t="inlineStr">
+      <c r="G111" s="13" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -10765,7 +10207,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q111" s="4" t="n"/>
       <c r="R111" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10855,7 +10296,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q112" s="4" t="n"/>
       <c r="R112" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -10945,7 +10385,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q113" s="4" t="n"/>
       <c r="R113" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -11035,7 +10474,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q114" s="4" t="n"/>
       <c r="R114" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -11125,7 +10563,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q115" s="4" t="n"/>
       <c r="R115" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -11215,7 +10652,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q116" s="4" t="n"/>
       <c r="R116" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -11305,7 +10741,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q117" s="4" t="n"/>
       <c r="R117" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -11343,7 +10778,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G118" s="14" t="inlineStr">
+      <c r="G118" s="13" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -11395,7 +10830,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q118" s="4" t="n"/>
       <c r="R118" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -11433,7 +10867,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G119" s="14" t="inlineStr">
+      <c r="G119" s="13" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -11485,7 +10919,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q119" s="4" t="n"/>
       <c r="R119" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -11575,7 +11008,6 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q120" s="4" t="n"/>
       <c r="R120" s="4" t="inlineStr">
         <is>
           <t>否</t>
@@ -11665,7 +11097,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q121" s="3" t="inlineStr">
+      <c r="Q121" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -11759,7 +11191,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q122" s="3" t="inlineStr">
+      <c r="Q122" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -11853,7 +11285,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q123" s="17" t="inlineStr">
+      <c r="Q123" s="21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -11876,7 +11308,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="3"/>
@@ -12165,7 +11597,7 @@
           <t>其他说明信息</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12179,7 +11611,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -12487,7 +11919,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>

</xml_diff>